<commit_message>
actualizacion del ejm excel con estMatriculados y de la bd con materias, docentes, etc de 2026 B
</commit_message>
<xml_diff>
--- a/src/main/resources/ejemploExcel/ejemplo.xlsx
+++ b/src/main/resources/ejemploExcel/ejemplo.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Daniel Alejandro\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B49EBC21-80FD-493D-AB46-6E70E1144868}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EA97FB3-A861-46CE-A3BF-C8029D981B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IQ y Agro" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913" iterateDelta="1E-4"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'IQ y Agro'!$A$1:$Q$365</definedName>
+  </definedNames>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1216,6 +1219,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:Q365"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1304,7 +1308,7 @@
         <v>8</v>
       </c>
       <c r="I2" s="2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
@@ -1347,7 +1351,7 @@
         <v>13</v>
       </c>
       <c r="I3" s="4">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J3" s="5">
         <v>46339</v>
@@ -1391,9 +1395,7 @@
         <v>22</v>
       </c>
       <c r="H4" s="2"/>
-      <c r="I4" s="2">
-        <v>0</v>
-      </c>
+      <c r="I4" s="2"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="3">
@@ -1435,7 +1437,7 @@
         <v>14</v>
       </c>
       <c r="I5" s="4">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -1480,7 +1482,7 @@
         <v>4</v>
       </c>
       <c r="I6" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
@@ -1497,7 +1499,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -1512,9 +1514,7 @@
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
-      <c r="I7" s="4">
-        <v>0</v>
-      </c>
+      <c r="I7" s="4"/>
       <c r="J7" s="4">
         <v>2</v>
       </c>
@@ -1561,9 +1561,7 @@
         <v>22</v>
       </c>
       <c r="H8" s="2"/>
-      <c r="I8" s="2">
-        <v>0</v>
-      </c>
+      <c r="I8" s="2"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2" t="s">
         <v>33</v>
@@ -1581,7 +1579,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -1596,9 +1594,7 @@
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
-      <c r="I9" s="4">
-        <v>0</v>
-      </c>
+      <c r="I9" s="4"/>
       <c r="J9" s="4">
         <v>0</v>
       </c>
@@ -1648,7 +1644,7 @@
         <v>13</v>
       </c>
       <c r="I10" s="2">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
@@ -1667,7 +1663,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -1682,9 +1678,7 @@
       <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
-      <c r="I11" s="4">
-        <v>0</v>
-      </c>
+      <c r="I11" s="4"/>
       <c r="J11" s="4">
         <v>0</v>
       </c>
@@ -1734,7 +1728,7 @@
         <v>15</v>
       </c>
       <c r="I12" s="2">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
@@ -1777,7 +1771,7 @@
         <v>15</v>
       </c>
       <c r="I13" s="4">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J13" s="4"/>
       <c r="K13" s="5">
@@ -1796,7 +1790,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1811,9 +1805,7 @@
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
-      <c r="I14" s="2">
-        <v>0</v>
-      </c>
+      <c r="I14" s="2"/>
       <c r="J14" s="2">
         <v>0</v>
       </c>
@@ -1863,7 +1855,7 @@
         <v>7</v>
       </c>
       <c r="I15" s="4">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J15" s="4"/>
       <c r="K15" s="5">
@@ -1906,7 +1898,7 @@
         <v>7</v>
       </c>
       <c r="I16" s="2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J16" s="2"/>
       <c r="K16" s="3">
@@ -1949,7 +1941,7 @@
         <v>7</v>
       </c>
       <c r="I17" s="4">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J17" s="4"/>
       <c r="K17" s="4"/>
@@ -1992,7 +1984,7 @@
         <v>8</v>
       </c>
       <c r="I18" s="2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
@@ -2035,7 +2027,7 @@
         <v>8</v>
       </c>
       <c r="I19" s="4">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J19" s="4"/>
       <c r="K19" s="4"/>
@@ -2078,7 +2070,7 @@
         <v>8</v>
       </c>
       <c r="I20" s="2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
@@ -2095,7 +2087,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4">
         <v>20</v>
       </c>
@@ -2110,9 +2102,7 @@
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
-      <c r="I21" s="4">
-        <v>0</v>
-      </c>
+      <c r="I21" s="4"/>
       <c r="J21" s="4">
         <v>0</v>
       </c>
@@ -2162,7 +2152,7 @@
         <v>3</v>
       </c>
       <c r="I22" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
@@ -2179,7 +2169,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="23" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4">
         <v>22</v>
       </c>
@@ -2194,9 +2184,7 @@
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
-      <c r="I23" s="4">
-        <v>0</v>
-      </c>
+      <c r="I23" s="4"/>
       <c r="J23" s="4">
         <v>0</v>
       </c>
@@ -2246,7 +2234,7 @@
         <v>40</v>
       </c>
       <c r="I24" s="2">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J24" s="3">
         <v>46212</v>
@@ -2265,7 +2253,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4">
         <v>24</v>
       </c>
@@ -2280,9 +2268,7 @@
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
-      <c r="I25" s="4">
-        <v>0</v>
-      </c>
+      <c r="I25" s="4"/>
       <c r="J25" s="4">
         <v>2</v>
       </c>
@@ -2332,7 +2318,7 @@
         <v>33</v>
       </c>
       <c r="I26" s="2">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="J26" s="2"/>
       <c r="K26" s="2" t="s">
@@ -2351,7 +2337,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="27" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4">
         <v>26</v>
       </c>
@@ -2366,9 +2352,7 @@
       <c r="F27" s="4"/>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
-      <c r="I27" s="4">
-        <v>0</v>
-      </c>
+      <c r="I27" s="4"/>
       <c r="J27" s="4">
         <v>0</v>
       </c>
@@ -2418,7 +2402,7 @@
         <v>45</v>
       </c>
       <c r="I28" s="2">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="J28" s="3">
         <v>46276</v>
@@ -2463,7 +2447,7 @@
         <v>45</v>
       </c>
       <c r="I29" s="4">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="J29" s="4" t="s">
         <v>33</v>
@@ -2482,7 +2466,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="30" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -2497,9 +2481,7 @@
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
-      <c r="I30" s="2">
-        <v>0</v>
-      </c>
+      <c r="I30" s="2"/>
       <c r="J30" s="2">
         <v>4</v>
       </c>
@@ -2549,7 +2531,7 @@
         <v>8</v>
       </c>
       <c r="I31" s="4">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J31" s="4"/>
       <c r="K31" s="4" t="s">
@@ -2592,7 +2574,7 @@
         <v>7</v>
       </c>
       <c r="I32" s="2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J32" s="2"/>
       <c r="K32" s="2" t="s">
@@ -2635,7 +2617,7 @@
         <v>3</v>
       </c>
       <c r="I33" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J33" s="4"/>
       <c r="K33" s="4"/>
@@ -2678,7 +2660,7 @@
         <v>3</v>
       </c>
       <c r="I34" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J34" s="3">
         <v>46212</v>
@@ -2725,7 +2707,7 @@
         <v>3</v>
       </c>
       <c r="I35" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J35" s="4"/>
       <c r="K35" s="4"/>
@@ -2742,7 +2724,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="36" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
         <v>35</v>
       </c>
@@ -2757,9 +2739,7 @@
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
-      <c r="I36" s="2">
-        <v>0</v>
-      </c>
+      <c r="I36" s="2"/>
       <c r="J36" s="2">
         <v>2</v>
       </c>
@@ -2809,7 +2789,7 @@
         <v>36</v>
       </c>
       <c r="I37" s="4">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="J37" s="4"/>
       <c r="K37" s="4"/>
@@ -2828,7 +2808,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="38" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
         <v>37</v>
       </c>
@@ -2843,9 +2823,7 @@
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
-      <c r="I38" s="2">
-        <v>0</v>
-      </c>
+      <c r="I38" s="2"/>
       <c r="J38" s="2">
         <v>0</v>
       </c>
@@ -2892,9 +2870,7 @@
         <v>22</v>
       </c>
       <c r="H39" s="4"/>
-      <c r="I39" s="4">
-        <v>0</v>
-      </c>
+      <c r="I39" s="4"/>
       <c r="J39" s="5">
         <v>46276</v>
       </c>
@@ -2914,7 +2890,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="40" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -2929,9 +2905,7 @@
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
-      <c r="I40" s="2">
-        <v>0</v>
-      </c>
+      <c r="I40" s="2"/>
       <c r="J40" s="2">
         <v>2</v>
       </c>
@@ -2978,9 +2952,7 @@
         <v>22</v>
       </c>
       <c r="H41" s="4"/>
-      <c r="I41" s="4">
-        <v>0</v>
-      </c>
+      <c r="I41" s="4"/>
       <c r="J41" s="4"/>
       <c r="K41" s="4" t="s">
         <v>34</v>
@@ -3022,7 +2994,7 @@
         <v>9</v>
       </c>
       <c r="I42" s="2">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J42" s="2"/>
       <c r="K42" s="2" t="s">
@@ -3041,7 +3013,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="43" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4">
         <v>42</v>
       </c>
@@ -3056,9 +3028,7 @@
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
-      <c r="I43" s="4">
-        <v>0</v>
-      </c>
+      <c r="I43" s="4"/>
       <c r="J43" s="4">
         <v>0</v>
       </c>
@@ -3108,7 +3078,7 @@
         <v>6</v>
       </c>
       <c r="I44" s="2">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J44" s="2" t="s">
         <v>33</v>
@@ -3151,7 +3121,7 @@
         <v>6</v>
       </c>
       <c r="I45" s="4">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J45" s="4" t="s">
         <v>44</v>
@@ -3194,7 +3164,7 @@
         <v>11</v>
       </c>
       <c r="I46" s="2">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
@@ -3234,9 +3204,7 @@
         <v>22</v>
       </c>
       <c r="H47" s="4"/>
-      <c r="I47" s="4">
-        <v>0</v>
-      </c>
+      <c r="I47" s="4"/>
       <c r="J47" s="4"/>
       <c r="K47" s="4"/>
       <c r="L47" s="4"/>
@@ -3278,7 +3246,7 @@
         <v>7</v>
       </c>
       <c r="I48" s="2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
@@ -3323,7 +3291,7 @@
         <v>6</v>
       </c>
       <c r="I49" s="4">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J49" s="4"/>
       <c r="K49" s="4" t="s">
@@ -3366,7 +3334,7 @@
         <v>7</v>
       </c>
       <c r="I50" s="2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J50" s="2"/>
       <c r="K50" s="2" t="s">
@@ -3409,7 +3377,7 @@
         <v>10</v>
       </c>
       <c r="I51" s="4">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J51" s="5">
         <v>46211</v>
@@ -3452,7 +3420,7 @@
         <v>10</v>
       </c>
       <c r="I52" s="2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J52" s="2"/>
       <c r="K52" s="3">
@@ -3495,7 +3463,7 @@
         <v>10</v>
       </c>
       <c r="I53" s="4">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J53" s="4"/>
       <c r="K53" s="4"/>
@@ -3538,7 +3506,7 @@
         <v>6</v>
       </c>
       <c r="I54" s="2">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J54" s="2"/>
       <c r="K54" s="2"/>
@@ -3581,7 +3549,7 @@
         <v>6</v>
       </c>
       <c r="I55" s="4">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J55" s="4"/>
       <c r="K55" s="4"/>
@@ -3598,7 +3566,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="56" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -3613,9 +3581,7 @@
       <c r="F56" s="2"/>
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
-      <c r="I56" s="2">
-        <v>0</v>
-      </c>
+      <c r="I56" s="2"/>
       <c r="J56" s="2">
         <v>5</v>
       </c>
@@ -3665,7 +3631,7 @@
         <v>3</v>
       </c>
       <c r="I57" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J57" s="4"/>
       <c r="K57" s="4"/>
@@ -3682,7 +3648,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="58" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -3697,9 +3663,7 @@
       <c r="F58" s="2"/>
       <c r="G58" s="2"/>
       <c r="H58" s="2"/>
-      <c r="I58" s="2">
-        <v>0</v>
-      </c>
+      <c r="I58" s="2"/>
       <c r="J58" s="2">
         <v>0</v>
       </c>
@@ -3749,7 +3713,7 @@
         <v>12</v>
       </c>
       <c r="I59" s="4">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J59" s="5">
         <v>46276</v>
@@ -3794,7 +3758,7 @@
         <v>13</v>
       </c>
       <c r="I60" s="2">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J60" s="3">
         <v>46339</v>
@@ -3836,9 +3800,7 @@
         <v>22</v>
       </c>
       <c r="H61" s="4"/>
-      <c r="I61" s="4">
-        <v>0</v>
-      </c>
+      <c r="I61" s="4"/>
       <c r="J61" s="4"/>
       <c r="K61" s="4"/>
       <c r="L61" s="4"/>
@@ -3880,7 +3842,7 @@
         <v>4</v>
       </c>
       <c r="I62" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J62" s="2"/>
       <c r="K62" s="2"/>
@@ -3897,7 +3859,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="63" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="4">
         <v>62</v>
       </c>
@@ -3912,9 +3874,7 @@
       <c r="F63" s="4"/>
       <c r="G63" s="4"/>
       <c r="H63" s="4"/>
-      <c r="I63" s="4">
-        <v>0</v>
-      </c>
+      <c r="I63" s="4"/>
       <c r="J63" s="4">
         <v>4</v>
       </c>
@@ -3964,7 +3924,7 @@
         <v>11</v>
       </c>
       <c r="I64" s="2">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J64" s="3">
         <v>46211</v>
@@ -4009,7 +3969,7 @@
         <v>10</v>
       </c>
       <c r="I65" s="4">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J65" s="4"/>
       <c r="K65" s="4"/>
@@ -4028,7 +3988,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="66" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -4043,9 +4003,7 @@
       <c r="F66" s="2"/>
       <c r="G66" s="2"/>
       <c r="H66" s="2"/>
-      <c r="I66" s="2">
-        <v>0</v>
-      </c>
+      <c r="I66" s="2"/>
       <c r="J66" s="2">
         <v>1</v>
       </c>
@@ -4092,9 +4050,7 @@
         <v>22</v>
       </c>
       <c r="H67" s="4"/>
-      <c r="I67" s="4">
-        <v>0</v>
-      </c>
+      <c r="I67" s="4"/>
       <c r="J67" s="4"/>
       <c r="K67" s="4" t="s">
         <v>33</v>
@@ -4136,7 +4092,7 @@
         <v>10</v>
       </c>
       <c r="I68" s="2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J68" s="2"/>
       <c r="K68" s="2" t="s">
@@ -4181,7 +4137,7 @@
         <v>6</v>
       </c>
       <c r="I69" s="4">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J69" s="4"/>
       <c r="K69" s="4"/>
@@ -4224,7 +4180,7 @@
         <v>7</v>
       </c>
       <c r="I70" s="2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J70" s="2"/>
       <c r="K70" s="2"/>
@@ -4241,7 +4197,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="71" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="4">
         <v>70</v>
       </c>
@@ -4256,9 +4212,7 @@
       <c r="F71" s="4"/>
       <c r="G71" s="4"/>
       <c r="H71" s="4"/>
-      <c r="I71" s="4">
-        <v>0</v>
-      </c>
+      <c r="I71" s="4"/>
       <c r="J71" s="4">
         <v>0</v>
       </c>
@@ -4308,7 +4262,7 @@
         <v>14</v>
       </c>
       <c r="I72" s="2">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="J72" s="3">
         <v>46243</v>
@@ -4327,7 +4281,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="73" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="4">
         <v>72</v>
       </c>
@@ -4342,9 +4296,7 @@
       <c r="F73" s="4"/>
       <c r="G73" s="4"/>
       <c r="H73" s="4"/>
-      <c r="I73" s="4">
-        <v>0</v>
-      </c>
+      <c r="I73" s="4"/>
       <c r="J73" s="4">
         <v>1</v>
       </c>
@@ -4394,7 +4346,7 @@
         <v>12</v>
       </c>
       <c r="I74" s="2">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J74" s="2"/>
       <c r="K74" s="2"/>
@@ -4437,7 +4389,7 @@
         <v>13</v>
       </c>
       <c r="I75" s="4">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J75" s="4"/>
       <c r="K75" s="4"/>
@@ -4480,7 +4432,7 @@
         <v>12</v>
       </c>
       <c r="I76" s="2">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J76" s="2" t="s">
         <v>33</v>
@@ -4499,7 +4451,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="77" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" s="4">
         <v>76</v>
       </c>
@@ -4514,9 +4466,7 @@
       <c r="F77" s="4"/>
       <c r="G77" s="4"/>
       <c r="H77" s="4"/>
-      <c r="I77" s="4">
-        <v>0</v>
-      </c>
+      <c r="I77" s="4"/>
       <c r="J77" s="4">
         <v>2</v>
       </c>
@@ -4566,7 +4516,7 @@
         <v>38</v>
       </c>
       <c r="I78" s="2">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="J78" s="2"/>
       <c r="K78" s="2"/>
@@ -4585,7 +4535,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="79" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79" s="4">
         <v>78</v>
       </c>
@@ -4600,9 +4550,7 @@
       <c r="F79" s="4"/>
       <c r="G79" s="4"/>
       <c r="H79" s="4"/>
-      <c r="I79" s="4">
-        <v>0</v>
-      </c>
+      <c r="I79" s="4"/>
       <c r="J79" s="4">
         <v>0</v>
       </c>
@@ -4649,9 +4597,7 @@
         <v>22</v>
       </c>
       <c r="H80" s="2"/>
-      <c r="I80" s="2">
-        <v>0</v>
-      </c>
+      <c r="I80" s="2"/>
       <c r="J80" s="2"/>
       <c r="K80" s="2"/>
       <c r="L80" s="2"/>
@@ -4669,7 +4615,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="81" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" s="4">
         <v>80</v>
       </c>
@@ -4684,9 +4630,7 @@
       <c r="F81" s="4"/>
       <c r="G81" s="4"/>
       <c r="H81" s="4"/>
-      <c r="I81" s="4">
-        <v>0</v>
-      </c>
+      <c r="I81" s="4"/>
       <c r="J81" s="4">
         <v>0</v>
       </c>
@@ -4736,7 +4680,7 @@
         <v>20</v>
       </c>
       <c r="I82" s="2">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J82" s="2"/>
       <c r="K82" s="2"/>
@@ -4778,9 +4722,7 @@
         <v>22</v>
       </c>
       <c r="H83" s="4"/>
-      <c r="I83" s="4">
-        <v>0</v>
-      </c>
+      <c r="I83" s="4"/>
       <c r="J83" s="5">
         <v>46276</v>
       </c>
@@ -4823,9 +4765,7 @@
         <v>22</v>
       </c>
       <c r="H84" s="2"/>
-      <c r="I84" s="2">
-        <v>0</v>
-      </c>
+      <c r="I84" s="2"/>
       <c r="J84" s="2"/>
       <c r="K84" s="2"/>
       <c r="L84" s="2"/>
@@ -4841,7 +4781,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="85" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" s="4">
         <v>84</v>
       </c>
@@ -4856,9 +4796,7 @@
       <c r="F85" s="4"/>
       <c r="G85" s="4"/>
       <c r="H85" s="4"/>
-      <c r="I85" s="4">
-        <v>0</v>
-      </c>
+      <c r="I85" s="4"/>
       <c r="J85" s="4">
         <v>2</v>
       </c>
@@ -4908,7 +4846,7 @@
         <v>45</v>
       </c>
       <c r="I86" s="2">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="J86" s="2" t="s">
         <v>33</v>
@@ -4927,7 +4865,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="87" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" s="4">
         <v>86</v>
       </c>
@@ -4942,9 +4880,7 @@
       <c r="F87" s="4"/>
       <c r="G87" s="4"/>
       <c r="H87" s="4"/>
-      <c r="I87" s="4">
-        <v>0</v>
-      </c>
+      <c r="I87" s="4"/>
       <c r="J87" s="4">
         <v>2</v>
       </c>
@@ -4994,7 +4930,7 @@
         <v>27</v>
       </c>
       <c r="I88" s="2">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="J88" s="2"/>
       <c r="K88" s="2" t="s">
@@ -5080,7 +5016,7 @@
         <v>20</v>
       </c>
       <c r="I90" s="2">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J90" s="2"/>
       <c r="K90" s="2"/>
@@ -5123,7 +5059,7 @@
         <v>20</v>
       </c>
       <c r="I91" s="4">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J91" s="4"/>
       <c r="K91" s="5">
@@ -5166,7 +5102,7 @@
         <v>20</v>
       </c>
       <c r="I92" s="2">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J92" s="3">
         <v>46276</v>
@@ -5209,7 +5145,7 @@
         <v>20</v>
       </c>
       <c r="I93" s="4">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J93" s="5">
         <v>46276</v>
@@ -5252,7 +5188,7 @@
         <v>22</v>
       </c>
       <c r="I94" s="2">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="J94" s="2"/>
       <c r="K94" s="2"/>
@@ -5295,7 +5231,7 @@
         <v>20</v>
       </c>
       <c r="I95" s="4">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J95" s="4"/>
       <c r="K95" s="4" t="s">
@@ -5338,7 +5274,7 @@
         <v>15</v>
       </c>
       <c r="I96" s="2">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J96" s="2"/>
       <c r="K96" s="2"/>
@@ -5381,7 +5317,7 @@
         <v>40</v>
       </c>
       <c r="I97" s="4">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J97" s="5">
         <v>46339</v>
@@ -5426,7 +5362,7 @@
         <v>40</v>
       </c>
       <c r="I98" s="2">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J98" s="3">
         <v>46339</v>
@@ -5553,7 +5489,7 @@
         <v>17</v>
       </c>
       <c r="I101" s="4">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="J101" s="5">
         <v>46211</v>
@@ -5600,7 +5536,7 @@
         <v>15</v>
       </c>
       <c r="I102" s="2">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J102" s="3">
         <v>46212</v>
@@ -5621,7 +5557,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="103" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" s="4">
         <v>102</v>
       </c>
@@ -5636,9 +5572,7 @@
       <c r="F103" s="4"/>
       <c r="G103" s="4"/>
       <c r="H103" s="4"/>
-      <c r="I103" s="4">
-        <v>0</v>
-      </c>
+      <c r="I103" s="4"/>
       <c r="J103" s="4">
         <v>11</v>
       </c>
@@ -5685,9 +5619,7 @@
         <v>22</v>
       </c>
       <c r="H104" s="2"/>
-      <c r="I104" s="2">
-        <v>0</v>
-      </c>
+      <c r="I104" s="2"/>
       <c r="J104" s="2"/>
       <c r="K104" s="2"/>
       <c r="L104" s="2"/>
@@ -5703,7 +5635,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="105" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" s="4">
         <v>104</v>
       </c>
@@ -5718,9 +5650,7 @@
       <c r="F105" s="4"/>
       <c r="G105" s="4"/>
       <c r="H105" s="4"/>
-      <c r="I105" s="4">
-        <v>0</v>
-      </c>
+      <c r="I105" s="4"/>
       <c r="J105" s="4">
         <v>0</v>
       </c>
@@ -5770,7 +5700,7 @@
         <v>10</v>
       </c>
       <c r="I106" s="2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J106" s="3">
         <v>46339</v>
@@ -5812,9 +5742,7 @@
         <v>22</v>
       </c>
       <c r="H107" s="4"/>
-      <c r="I107" s="4">
-        <v>0</v>
-      </c>
+      <c r="I107" s="4"/>
       <c r="J107" s="4"/>
       <c r="K107" s="4"/>
       <c r="L107" s="4"/>
@@ -5830,7 +5758,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="108" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" s="2">
         <v>107</v>
       </c>
@@ -5845,9 +5773,7 @@
       <c r="F108" s="2"/>
       <c r="G108" s="2"/>
       <c r="H108" s="2"/>
-      <c r="I108" s="2">
-        <v>0</v>
-      </c>
+      <c r="I108" s="2"/>
       <c r="J108" s="2">
         <v>2</v>
       </c>
@@ -5897,7 +5823,7 @@
         <v>3</v>
       </c>
       <c r="I109" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J109" s="4"/>
       <c r="K109" s="4" t="s">
@@ -5940,7 +5866,7 @@
         <v>20</v>
       </c>
       <c r="I110" s="2">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J110" s="3">
         <v>46244</v>
@@ -5983,7 +5909,7 @@
         <v>28</v>
       </c>
       <c r="I111" s="4">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="J111" s="5">
         <v>46339</v>
@@ -6026,7 +5952,7 @@
         <v>27</v>
       </c>
       <c r="I112" s="2">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="J112" s="2" t="s">
         <v>33</v>
@@ -6043,7 +5969,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="113" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" s="4">
         <v>112</v>
       </c>
@@ -6058,9 +5984,7 @@
       <c r="F113" s="4"/>
       <c r="G113" s="4"/>
       <c r="H113" s="4"/>
-      <c r="I113" s="4">
-        <v>0</v>
-      </c>
+      <c r="I113" s="4"/>
       <c r="J113" s="4">
         <v>6</v>
       </c>
@@ -6110,7 +6034,7 @@
         <v>15</v>
       </c>
       <c r="I114" s="2">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J114" s="2"/>
       <c r="K114" s="3">
@@ -6153,7 +6077,7 @@
         <v>3</v>
       </c>
       <c r="I115" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J115" s="4"/>
       <c r="K115" s="5">
@@ -6198,7 +6122,7 @@
         <v>16</v>
       </c>
       <c r="I116" s="2">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="J116" s="3">
         <v>46276</v>
@@ -6217,7 +6141,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="117" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" s="4">
         <v>116</v>
       </c>
@@ -6232,9 +6156,7 @@
       <c r="F117" s="4"/>
       <c r="G117" s="4"/>
       <c r="H117" s="4"/>
-      <c r="I117" s="4">
-        <v>0</v>
-      </c>
+      <c r="I117" s="4"/>
       <c r="J117" s="4">
         <v>2</v>
       </c>
@@ -6284,7 +6206,7 @@
         <v>46</v>
       </c>
       <c r="I118" s="2">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="J118" s="2"/>
       <c r="K118" s="3">
@@ -6303,7 +6225,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="119" spans="1:17" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:17" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" s="4">
         <v>118</v>
       </c>
@@ -6318,9 +6240,7 @@
       <c r="F119" s="4"/>
       <c r="G119" s="4"/>
       <c r="H119" s="4"/>
-      <c r="I119" s="4">
-        <v>0</v>
-      </c>
+      <c r="I119" s="4"/>
       <c r="J119" s="4">
         <v>0</v>
       </c>
@@ -6370,7 +6290,7 @@
         <v>28</v>
       </c>
       <c r="I120" s="2">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="J120" s="3">
         <v>46276</v>
@@ -6417,7 +6337,7 @@
         <v>40</v>
       </c>
       <c r="I121" s="4">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J121" s="4"/>
       <c r="K121" s="5">
@@ -6462,7 +6382,7 @@
         <v>40</v>
       </c>
       <c r="I122" s="2">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J122" s="2"/>
       <c r="K122" s="2"/>
@@ -6481,7 +6401,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="123" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" s="4">
         <v>4</v>
       </c>
@@ -6496,9 +6416,7 @@
       <c r="F123" s="4"/>
       <c r="G123" s="4"/>
       <c r="H123" s="4"/>
-      <c r="I123" s="4">
-        <v>0</v>
-      </c>
+      <c r="I123" s="4"/>
       <c r="J123" s="4">
         <v>2</v>
       </c>
@@ -6548,7 +6466,7 @@
         <v>2</v>
       </c>
       <c r="I124" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J124" s="2"/>
       <c r="K124" s="2"/>
@@ -6591,7 +6509,7 @@
         <v>40</v>
       </c>
       <c r="I125" s="4">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J125" s="4"/>
       <c r="K125" s="4"/>
@@ -6634,7 +6552,7 @@
         <v>3</v>
       </c>
       <c r="I126" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J126" s="2"/>
       <c r="K126" s="2"/>
@@ -6651,7 +6569,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="127" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" s="4">
         <v>8</v>
       </c>
@@ -6666,9 +6584,7 @@
       <c r="F127" s="4"/>
       <c r="G127" s="4"/>
       <c r="H127" s="4"/>
-      <c r="I127" s="4">
-        <v>0</v>
-      </c>
+      <c r="I127" s="4"/>
       <c r="J127" s="4">
         <v>0</v>
       </c>
@@ -6718,7 +6634,7 @@
         <v>30</v>
       </c>
       <c r="I128" s="2">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J128" s="2"/>
       <c r="K128" s="2" t="s">
@@ -6735,7 +6651,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="129" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" s="4">
         <v>10</v>
       </c>
@@ -6750,9 +6666,7 @@
       <c r="F129" s="4"/>
       <c r="G129" s="4"/>
       <c r="H129" s="4"/>
-      <c r="I129" s="4">
-        <v>0</v>
-      </c>
+      <c r="I129" s="4"/>
       <c r="J129" s="4">
         <v>0</v>
       </c>
@@ -6802,7 +6716,7 @@
         <v>30</v>
       </c>
       <c r="I130" s="2">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J130" s="2"/>
       <c r="K130" s="2"/>
@@ -6819,7 +6733,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="131" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" s="4">
         <v>12</v>
       </c>
@@ -6834,9 +6748,7 @@
       <c r="F131" s="4"/>
       <c r="G131" s="4"/>
       <c r="H131" s="4"/>
-      <c r="I131" s="4">
-        <v>0</v>
-      </c>
+      <c r="I131" s="4"/>
       <c r="J131" s="4">
         <v>0</v>
       </c>
@@ -6886,7 +6798,7 @@
         <v>8</v>
       </c>
       <c r="I132" s="2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J132" s="2"/>
       <c r="K132" s="2"/>
@@ -6929,7 +6841,7 @@
         <v>8</v>
       </c>
       <c r="I133" s="4">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J133" s="4"/>
       <c r="K133" s="4"/>
@@ -6972,7 +6884,7 @@
         <v>8</v>
       </c>
       <c r="I134" s="2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J134" s="2"/>
       <c r="K134" s="2"/>
@@ -7015,7 +6927,7 @@
         <v>8</v>
       </c>
       <c r="I135" s="4">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J135" s="4"/>
       <c r="K135" s="4"/>
@@ -7058,7 +6970,7 @@
         <v>8</v>
       </c>
       <c r="I136" s="2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J136" s="2"/>
       <c r="K136" s="2"/>
@@ -7101,7 +7013,7 @@
         <v>8</v>
       </c>
       <c r="I137" s="4">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J137" s="4"/>
       <c r="K137" s="4"/>
@@ -7144,7 +7056,7 @@
         <v>12</v>
       </c>
       <c r="I138" s="2">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J138" s="2"/>
       <c r="K138" s="2"/>
@@ -7187,7 +7099,7 @@
         <v>12</v>
       </c>
       <c r="I139" s="4">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J139" s="4"/>
       <c r="K139" s="4"/>
@@ -7230,7 +7142,7 @@
         <v>12</v>
       </c>
       <c r="I140" s="2">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J140" s="2"/>
       <c r="K140" s="2"/>
@@ -7273,7 +7185,7 @@
         <v>9</v>
       </c>
       <c r="I141" s="4">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J141" s="4"/>
       <c r="K141" s="4"/>
@@ -7316,7 +7228,7 @@
         <v>9</v>
       </c>
       <c r="I142" s="2">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J142" s="2"/>
       <c r="K142" s="2"/>
@@ -7359,7 +7271,7 @@
         <v>9</v>
       </c>
       <c r="I143" s="4">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J143" s="4"/>
       <c r="K143" s="4"/>
@@ -7402,7 +7314,7 @@
         <v>9</v>
       </c>
       <c r="I144" s="2">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J144" s="2"/>
       <c r="K144" s="2"/>
@@ -7445,7 +7357,7 @@
         <v>9</v>
       </c>
       <c r="I145" s="4">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J145" s="4" t="s">
         <v>72</v>
@@ -7488,7 +7400,7 @@
         <v>9</v>
       </c>
       <c r="I146" s="2">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J146" s="2" t="s">
         <v>34</v>
@@ -7531,7 +7443,7 @@
         <v>9</v>
       </c>
       <c r="I147" s="4">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J147" s="4" t="s">
         <v>78</v>
@@ -7574,7 +7486,7 @@
         <v>9</v>
       </c>
       <c r="I148" s="2">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J148" s="2" t="s">
         <v>68</v>
@@ -7591,7 +7503,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="149" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" s="4">
         <v>30</v>
       </c>
@@ -7606,9 +7518,7 @@
       <c r="F149" s="4"/>
       <c r="G149" s="4"/>
       <c r="H149" s="4"/>
-      <c r="I149" s="4">
-        <v>0</v>
-      </c>
+      <c r="I149" s="4"/>
       <c r="J149" s="4">
         <v>4</v>
       </c>
@@ -7658,7 +7568,7 @@
         <v>40</v>
       </c>
       <c r="I150" s="2">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J150" s="2"/>
       <c r="K150" s="2"/>
@@ -7703,7 +7613,7 @@
         <v>20</v>
       </c>
       <c r="I151" s="4">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J151" s="4"/>
       <c r="K151" s="4"/>
@@ -7746,7 +7656,7 @@
         <v>3</v>
       </c>
       <c r="I152" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J152" s="2"/>
       <c r="K152" s="2"/>
@@ -7789,7 +7699,7 @@
         <v>22</v>
       </c>
       <c r="I153" s="4">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="J153" s="4"/>
       <c r="K153" s="5">
@@ -7808,7 +7718,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="154" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" s="2">
         <v>35</v>
       </c>
@@ -7823,9 +7733,7 @@
       <c r="F154" s="2"/>
       <c r="G154" s="2"/>
       <c r="H154" s="2"/>
-      <c r="I154" s="2">
-        <v>0</v>
-      </c>
+      <c r="I154" s="2"/>
       <c r="J154" s="2">
         <v>0</v>
       </c>
@@ -7872,9 +7780,7 @@
         <v>22</v>
       </c>
       <c r="H155" s="4"/>
-      <c r="I155" s="4">
-        <v>0</v>
-      </c>
+      <c r="I155" s="4"/>
       <c r="J155" s="4"/>
       <c r="K155" s="4" t="s">
         <v>104</v>
@@ -7917,9 +7823,7 @@
         <v>22</v>
       </c>
       <c r="H156" s="2"/>
-      <c r="I156" s="2">
-        <v>0</v>
-      </c>
+      <c r="I156" s="2"/>
       <c r="J156" s="2"/>
       <c r="K156" s="3">
         <v>46276</v>
@@ -7965,7 +7869,7 @@
         <v>3</v>
       </c>
       <c r="I157" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J157" s="4"/>
       <c r="K157" s="4"/>
@@ -7982,7 +7886,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="158" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" s="2">
         <v>39</v>
       </c>
@@ -7997,9 +7901,7 @@
       <c r="F158" s="2"/>
       <c r="G158" s="2"/>
       <c r="H158" s="2"/>
-      <c r="I158" s="2">
-        <v>0</v>
-      </c>
+      <c r="I158" s="2"/>
       <c r="J158" s="2">
         <v>0</v>
       </c>
@@ -8049,7 +7951,7 @@
         <v>46</v>
       </c>
       <c r="I159" s="4">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="J159" s="4"/>
       <c r="K159" s="4"/>
@@ -8092,7 +7994,7 @@
         <v>40</v>
       </c>
       <c r="I160" s="2">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J160" s="2"/>
       <c r="K160" s="2"/>
@@ -8109,7 +8011,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="161" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" s="4">
         <v>42</v>
       </c>
@@ -8124,9 +8026,7 @@
       <c r="F161" s="4"/>
       <c r="G161" s="4"/>
       <c r="H161" s="4"/>
-      <c r="I161" s="4">
-        <v>0</v>
-      </c>
+      <c r="I161" s="4"/>
       <c r="J161" s="4">
         <v>0</v>
       </c>
@@ -8176,7 +8076,7 @@
         <v>7</v>
       </c>
       <c r="I162" s="2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J162" s="2" t="s">
         <v>78</v>
@@ -8219,7 +8119,7 @@
         <v>7</v>
       </c>
       <c r="I163" s="4">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J163" s="4" t="s">
         <v>68</v>
@@ -8262,7 +8162,7 @@
         <v>7</v>
       </c>
       <c r="I164" s="2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J164" s="2" t="s">
         <v>72</v>
@@ -8305,7 +8205,7 @@
         <v>7</v>
       </c>
       <c r="I165" s="4">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J165" s="4" t="s">
         <v>34</v>
@@ -8322,7 +8222,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="166" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" s="2">
         <v>47</v>
       </c>
@@ -8337,9 +8237,7 @@
       <c r="F166" s="2"/>
       <c r="G166" s="2"/>
       <c r="H166" s="2"/>
-      <c r="I166" s="2">
-        <v>0</v>
-      </c>
+      <c r="I166" s="2"/>
       <c r="J166" s="2">
         <v>4</v>
       </c>
@@ -8389,7 +8287,7 @@
         <v>38</v>
       </c>
       <c r="I167" s="4">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="J167" s="5">
         <v>46243</v>
@@ -8434,7 +8332,7 @@
         <v>25</v>
       </c>
       <c r="I168" s="2">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="J168" s="2"/>
       <c r="K168" s="2" t="s">
@@ -8453,7 +8351,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="169" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" s="4">
         <v>50</v>
       </c>
@@ -8468,9 +8366,7 @@
       <c r="F169" s="4"/>
       <c r="G169" s="4"/>
       <c r="H169" s="4"/>
-      <c r="I169" s="4">
-        <v>0</v>
-      </c>
+      <c r="I169" s="4"/>
       <c r="J169" s="4">
         <v>1</v>
       </c>
@@ -8520,7 +8416,7 @@
         <v>40</v>
       </c>
       <c r="I170" s="2">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J170" s="2"/>
       <c r="K170" s="3">
@@ -8565,7 +8461,7 @@
         <v>41</v>
       </c>
       <c r="I171" s="4">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="J171" s="5">
         <v>46276</v>
@@ -8584,7 +8480,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="172" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" s="2">
         <v>53</v>
       </c>
@@ -8599,9 +8495,7 @@
       <c r="F172" s="2"/>
       <c r="G172" s="2"/>
       <c r="H172" s="2"/>
-      <c r="I172" s="2">
-        <v>0</v>
-      </c>
+      <c r="I172" s="2"/>
       <c r="J172" s="2">
         <v>2</v>
       </c>
@@ -8651,7 +8545,7 @@
         <v>35</v>
       </c>
       <c r="I173" s="4">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="J173" s="5">
         <v>46339</v>
@@ -8696,7 +8590,7 @@
         <v>3</v>
       </c>
       <c r="I174" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J174" s="2"/>
       <c r="K174" s="2"/>
@@ -8713,7 +8607,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="175" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" s="4">
         <v>56</v>
       </c>
@@ -8728,9 +8622,7 @@
       <c r="F175" s="4"/>
       <c r="G175" s="4"/>
       <c r="H175" s="4"/>
-      <c r="I175" s="4">
-        <v>0</v>
-      </c>
+      <c r="I175" s="4"/>
       <c r="J175" s="4">
         <v>2</v>
       </c>
@@ -8780,7 +8672,7 @@
         <v>30</v>
       </c>
       <c r="I176" s="2">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J176" s="3">
         <v>46306</v>
@@ -8825,7 +8717,7 @@
         <v>40</v>
       </c>
       <c r="I177" s="4">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J177" s="4"/>
       <c r="K177" s="5">
@@ -8844,7 +8736,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="178" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" s="2">
         <v>59</v>
       </c>
@@ -8859,9 +8751,7 @@
       <c r="F178" s="2"/>
       <c r="G178" s="2"/>
       <c r="H178" s="2"/>
-      <c r="I178" s="2">
-        <v>0</v>
-      </c>
+      <c r="I178" s="2"/>
       <c r="J178" s="2">
         <v>1</v>
       </c>
@@ -8911,7 +8801,7 @@
         <v>2</v>
       </c>
       <c r="I179" s="4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J179" s="4"/>
       <c r="K179" s="4"/>
@@ -8954,7 +8844,7 @@
         <v>30</v>
       </c>
       <c r="I180" s="2">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J180" s="2"/>
       <c r="K180" s="3">
@@ -8999,7 +8889,7 @@
         <v>3</v>
       </c>
       <c r="I181" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J181" s="4"/>
       <c r="K181" s="4"/>
@@ -9016,7 +8906,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="182" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" s="2">
         <v>63</v>
       </c>
@@ -9031,9 +8921,7 @@
       <c r="F182" s="2"/>
       <c r="G182" s="2"/>
       <c r="H182" s="2"/>
-      <c r="I182" s="2">
-        <v>0</v>
-      </c>
+      <c r="I182" s="2"/>
       <c r="J182" s="2">
         <v>0</v>
       </c>
@@ -9083,7 +8971,7 @@
         <v>24</v>
       </c>
       <c r="I183" s="4">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="J183" s="4"/>
       <c r="K183" s="4" t="s">
@@ -9125,9 +9013,7 @@
         <v>22</v>
       </c>
       <c r="H184" s="2"/>
-      <c r="I184" s="2">
-        <v>0</v>
-      </c>
+      <c r="I184" s="2"/>
       <c r="J184" s="2"/>
       <c r="K184" s="3">
         <v>46276</v>
@@ -9173,7 +9059,7 @@
         <v>48</v>
       </c>
       <c r="I185" s="4">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="J185" s="5">
         <v>46339</v>
@@ -9194,7 +9080,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="186" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186" s="2">
         <v>67</v>
       </c>
@@ -9209,9 +9095,7 @@
       <c r="F186" s="2"/>
       <c r="G186" s="2"/>
       <c r="H186" s="2"/>
-      <c r="I186" s="2">
-        <v>0</v>
-      </c>
+      <c r="I186" s="2"/>
       <c r="J186" s="2">
         <v>2</v>
       </c>
@@ -9261,7 +9145,7 @@
         <v>40</v>
       </c>
       <c r="I187" s="4">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J187" s="4"/>
       <c r="K187" s="4"/>
@@ -9278,7 +9162,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="188" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" s="2">
         <v>69</v>
       </c>
@@ -9293,9 +9177,7 @@
       <c r="F188" s="2"/>
       <c r="G188" s="2"/>
       <c r="H188" s="2"/>
-      <c r="I188" s="2">
-        <v>0</v>
-      </c>
+      <c r="I188" s="2"/>
       <c r="J188" s="2">
         <v>0</v>
       </c>
@@ -9345,7 +9227,7 @@
         <v>2</v>
       </c>
       <c r="I189" s="4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J189" s="4"/>
       <c r="K189" s="4"/>
@@ -9362,7 +9244,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="190" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" s="2">
         <v>71</v>
       </c>
@@ -9377,9 +9259,7 @@
       <c r="F190" s="2"/>
       <c r="G190" s="2"/>
       <c r="H190" s="2"/>
-      <c r="I190" s="2">
-        <v>0</v>
-      </c>
+      <c r="I190" s="2"/>
       <c r="J190" s="2">
         <v>0</v>
       </c>
@@ -9429,7 +9309,7 @@
         <v>52</v>
       </c>
       <c r="I191" s="4">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="J191" s="4"/>
       <c r="K191" s="4"/>
@@ -9474,7 +9354,7 @@
         <v>24</v>
       </c>
       <c r="I192" s="2">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="J192" s="2"/>
       <c r="K192" s="2" t="s">
@@ -9493,7 +9373,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="193" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" s="4">
         <v>74</v>
       </c>
@@ -9508,9 +9388,7 @@
       <c r="F193" s="4"/>
       <c r="G193" s="4"/>
       <c r="H193" s="4"/>
-      <c r="I193" s="4">
-        <v>0</v>
-      </c>
+      <c r="I193" s="4"/>
       <c r="J193" s="4">
         <v>0</v>
       </c>
@@ -9560,7 +9438,7 @@
         <v>40</v>
       </c>
       <c r="I194" s="2">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J194" s="2" t="s">
         <v>33</v>
@@ -9577,7 +9455,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="195" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195" s="4">
         <v>76</v>
       </c>
@@ -9592,9 +9470,7 @@
       <c r="F195" s="4"/>
       <c r="G195" s="4"/>
       <c r="H195" s="4"/>
-      <c r="I195" s="4">
-        <v>0</v>
-      </c>
+      <c r="I195" s="4"/>
       <c r="J195" s="4">
         <v>2</v>
       </c>
@@ -9644,7 +9520,7 @@
         <v>3</v>
       </c>
       <c r="I196" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J196" s="2"/>
       <c r="K196" s="2"/>
@@ -9684,9 +9560,7 @@
         <v>22</v>
       </c>
       <c r="H197" s="4"/>
-      <c r="I197" s="4">
-        <v>0</v>
-      </c>
+      <c r="I197" s="4"/>
       <c r="J197" s="4"/>
       <c r="K197" s="4"/>
       <c r="L197" s="4"/>
@@ -9728,7 +9602,7 @@
         <v>3</v>
       </c>
       <c r="I198" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J198" s="2"/>
       <c r="K198" s="2"/>
@@ -9771,7 +9645,7 @@
         <v>40</v>
       </c>
       <c r="I199" s="4">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J199" s="5">
         <v>46276</v>
@@ -9816,7 +9690,7 @@
         <v>40</v>
       </c>
       <c r="I200" s="2">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J200" s="3">
         <v>46339</v>
@@ -9835,7 +9709,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="201" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" s="4">
         <v>82</v>
       </c>
@@ -9850,9 +9724,7 @@
       <c r="F201" s="4"/>
       <c r="G201" s="4"/>
       <c r="H201" s="4"/>
-      <c r="I201" s="4">
-        <v>0</v>
-      </c>
+      <c r="I201" s="4"/>
       <c r="J201" s="4">
         <v>4</v>
       </c>
@@ -9902,7 +9774,7 @@
         <v>22</v>
       </c>
       <c r="I202" s="2">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="J202" s="2"/>
       <c r="K202" s="3">
@@ -9949,7 +9821,7 @@
         <v>3</v>
       </c>
       <c r="I203" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J203" s="4"/>
       <c r="K203" s="4"/>
@@ -9992,7 +9864,7 @@
         <v>3</v>
       </c>
       <c r="I204" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J204" s="2"/>
       <c r="K204" s="2"/>
@@ -10009,7 +9881,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="205" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205" s="4">
         <v>86</v>
       </c>
@@ -10024,9 +9896,7 @@
       <c r="F205" s="4"/>
       <c r="G205" s="4"/>
       <c r="H205" s="4"/>
-      <c r="I205" s="4">
-        <v>0</v>
-      </c>
+      <c r="I205" s="4"/>
       <c r="J205" s="4">
         <v>0</v>
       </c>
@@ -10073,9 +9943,7 @@
         <v>22</v>
       </c>
       <c r="H206" s="2"/>
-      <c r="I206" s="2">
-        <v>0</v>
-      </c>
+      <c r="I206" s="2"/>
       <c r="J206" s="2"/>
       <c r="K206" s="3">
         <v>46212</v>
@@ -10117,7 +9985,7 @@
         <v>7</v>
       </c>
       <c r="I207" s="4">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J207" s="4"/>
       <c r="K207" s="4"/>
@@ -10160,7 +10028,7 @@
         <v>11</v>
       </c>
       <c r="I208" s="2">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J208" s="2"/>
       <c r="K208" s="2"/>
@@ -10200,9 +10068,7 @@
         <v>22</v>
       </c>
       <c r="H209" s="4"/>
-      <c r="I209" s="4">
-        <v>0</v>
-      </c>
+      <c r="I209" s="4"/>
       <c r="J209" s="4"/>
       <c r="K209" s="4"/>
       <c r="L209" s="4"/>
@@ -10244,7 +10110,7 @@
         <v>13</v>
       </c>
       <c r="I210" s="2">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J210" s="2"/>
       <c r="K210" s="3">
@@ -10286,9 +10152,7 @@
         <v>22</v>
       </c>
       <c r="H211" s="4"/>
-      <c r="I211" s="4">
-        <v>0</v>
-      </c>
+      <c r="I211" s="4"/>
       <c r="J211" s="4" t="s">
         <v>72</v>
       </c>
@@ -10330,7 +10194,7 @@
         <v>12</v>
       </c>
       <c r="I212" s="2">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J212" s="2" t="s">
         <v>34</v>
@@ -10372,9 +10236,7 @@
         <v>22</v>
       </c>
       <c r="H213" s="4"/>
-      <c r="I213" s="4">
-        <v>0</v>
-      </c>
+      <c r="I213" s="4"/>
       <c r="J213" s="4"/>
       <c r="K213" s="4"/>
       <c r="L213" s="4" t="s">
@@ -10416,7 +10278,7 @@
         <v>14</v>
       </c>
       <c r="I214" s="2">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="J214" s="3">
         <v>46369</v>
@@ -10435,7 +10297,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="215" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215" s="4">
         <v>96</v>
       </c>
@@ -10450,9 +10312,7 @@
       <c r="F215" s="4"/>
       <c r="G215" s="4"/>
       <c r="H215" s="4"/>
-      <c r="I215" s="4">
-        <v>0</v>
-      </c>
+      <c r="I215" s="4"/>
       <c r="J215" s="4">
         <v>3</v>
       </c>
@@ -10502,7 +10362,7 @@
         <v>3</v>
       </c>
       <c r="I216" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J216" s="2"/>
       <c r="K216" s="2"/>
@@ -10542,9 +10402,7 @@
         <v>22</v>
       </c>
       <c r="H217" s="4"/>
-      <c r="I217" s="4">
-        <v>0</v>
-      </c>
+      <c r="I217" s="4"/>
       <c r="J217" s="4"/>
       <c r="K217" s="5">
         <v>46369</v>
@@ -10583,9 +10441,7 @@
         <v>22</v>
       </c>
       <c r="H218" s="2"/>
-      <c r="I218" s="2">
-        <v>0</v>
-      </c>
+      <c r="I218" s="2"/>
       <c r="J218" s="3">
         <v>46369</v>
       </c>
@@ -10627,7 +10483,7 @@
         <v>26</v>
       </c>
       <c r="I219" s="4">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="J219" s="4"/>
       <c r="K219" s="5">
@@ -10672,7 +10528,7 @@
         <v>29</v>
       </c>
       <c r="I220" s="2">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="J220" s="3">
         <v>46338</v>
@@ -10717,7 +10573,7 @@
         <v>15</v>
       </c>
       <c r="I221" s="4">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J221" s="4"/>
       <c r="K221" s="4"/>
@@ -10734,7 +10590,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="222" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A222" s="2">
         <v>103</v>
       </c>
@@ -10749,9 +10605,7 @@
       <c r="F222" s="2"/>
       <c r="G222" s="2"/>
       <c r="H222" s="2"/>
-      <c r="I222" s="2">
-        <v>0</v>
-      </c>
+      <c r="I222" s="2"/>
       <c r="J222" s="2">
         <v>2</v>
       </c>
@@ -10801,7 +10655,7 @@
         <v>30</v>
       </c>
       <c r="I223" s="4">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J223" s="4"/>
       <c r="K223" s="4"/>
@@ -10846,7 +10700,7 @@
         <v>40</v>
       </c>
       <c r="I224" s="2">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J224" s="2"/>
       <c r="K224" s="2"/>
@@ -10889,7 +10743,7 @@
         <v>3</v>
       </c>
       <c r="I225" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J225" s="4"/>
       <c r="K225" s="4"/>
@@ -10906,7 +10760,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="226" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A226" s="2">
         <v>107</v>
       </c>
@@ -10921,9 +10775,7 @@
       <c r="F226" s="2"/>
       <c r="G226" s="2"/>
       <c r="H226" s="2"/>
-      <c r="I226" s="2">
-        <v>0</v>
-      </c>
+      <c r="I226" s="2"/>
       <c r="J226" s="2">
         <v>0</v>
       </c>
@@ -10973,7 +10825,7 @@
         <v>40</v>
       </c>
       <c r="I227" s="4">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J227" s="4"/>
       <c r="K227" s="4"/>
@@ -11016,7 +10868,7 @@
         <v>38</v>
       </c>
       <c r="I228" s="2">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="J228" s="2" t="s">
         <v>33</v>
@@ -11033,7 +10885,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="229" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A229" s="4">
         <v>110</v>
       </c>
@@ -11048,9 +10900,7 @@
       <c r="F229" s="4"/>
       <c r="G229" s="4"/>
       <c r="H229" s="4"/>
-      <c r="I229" s="4">
-        <v>0</v>
-      </c>
+      <c r="I229" s="4"/>
       <c r="J229" s="4">
         <v>2</v>
       </c>
@@ -11100,7 +10950,7 @@
         <v>37</v>
       </c>
       <c r="I230" s="2">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="J230" s="3">
         <v>46243</v>
@@ -11119,7 +10969,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="231" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A231" s="4">
         <v>112</v>
       </c>
@@ -11134,9 +10984,7 @@
       <c r="F231" s="4"/>
       <c r="G231" s="4"/>
       <c r="H231" s="4"/>
-      <c r="I231" s="4">
-        <v>0</v>
-      </c>
+      <c r="I231" s="4"/>
       <c r="J231" s="4">
         <v>1</v>
       </c>
@@ -11186,7 +11034,7 @@
         <v>7</v>
       </c>
       <c r="I232" s="2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J232" s="2" t="s">
         <v>72</v>
@@ -11229,7 +11077,7 @@
         <v>7</v>
       </c>
       <c r="I233" s="4">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J233" s="4" t="s">
         <v>34</v>
@@ -11272,7 +11120,7 @@
         <v>7</v>
       </c>
       <c r="I234" s="2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J234" s="2" t="s">
         <v>78</v>
@@ -11315,7 +11163,7 @@
         <v>7</v>
       </c>
       <c r="I235" s="4">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J235" s="4" t="s">
         <v>68</v>
@@ -11358,7 +11206,7 @@
         <v>6</v>
       </c>
       <c r="I236" s="2">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J236" s="2"/>
       <c r="K236" s="2"/>
@@ -11401,7 +11249,7 @@
         <v>6</v>
       </c>
       <c r="I237" s="4">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J237" s="4"/>
       <c r="K237" s="4"/>
@@ -11418,7 +11266,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="238" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A238" s="2">
         <v>119</v>
       </c>
@@ -11433,9 +11281,7 @@
       <c r="F238" s="2"/>
       <c r="G238" s="2"/>
       <c r="H238" s="2"/>
-      <c r="I238" s="2">
-        <v>0</v>
-      </c>
+      <c r="I238" s="2"/>
       <c r="J238" s="2">
         <v>4</v>
       </c>
@@ -11482,9 +11328,7 @@
         <v>22</v>
       </c>
       <c r="H239" s="4"/>
-      <c r="I239" s="4">
-        <v>0</v>
-      </c>
+      <c r="I239" s="4"/>
       <c r="J239" s="4"/>
       <c r="K239" s="4" t="s">
         <v>104</v>
@@ -11530,7 +11374,7 @@
         <v>3</v>
       </c>
       <c r="I240" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J240" s="2"/>
       <c r="K240" s="2"/>
@@ -11573,7 +11417,7 @@
         <v>3</v>
       </c>
       <c r="I241" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J241" s="4"/>
       <c r="K241" s="4"/>
@@ -11590,7 +11434,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="242" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A242" s="2">
         <v>123</v>
       </c>
@@ -11605,9 +11449,7 @@
       <c r="F242" s="2"/>
       <c r="G242" s="2"/>
       <c r="H242" s="2"/>
-      <c r="I242" s="2">
-        <v>0</v>
-      </c>
+      <c r="I242" s="2"/>
       <c r="J242" s="2">
         <v>0</v>
       </c>
@@ -11657,7 +11499,7 @@
         <v>40</v>
       </c>
       <c r="I243" s="4">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J243" s="4"/>
       <c r="K243" s="4" t="s">
@@ -11676,7 +11518,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="244" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A244" s="2">
         <v>125</v>
       </c>
@@ -11691,9 +11533,7 @@
       <c r="F244" s="2"/>
       <c r="G244" s="2"/>
       <c r="H244" s="2"/>
-      <c r="I244" s="2">
-        <v>0</v>
-      </c>
+      <c r="I244" s="2"/>
       <c r="J244" s="2">
         <v>0</v>
       </c>
@@ -11740,9 +11580,7 @@
         <v>22</v>
       </c>
       <c r="H245" s="4"/>
-      <c r="I245" s="4">
-        <v>0</v>
-      </c>
+      <c r="I245" s="4"/>
       <c r="J245" s="4"/>
       <c r="K245" s="4"/>
       <c r="L245" s="4" t="s">
@@ -11788,7 +11626,7 @@
         <v>3</v>
       </c>
       <c r="I246" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J246" s="2"/>
       <c r="K246" s="2"/>
@@ -11831,7 +11669,7 @@
         <v>35</v>
       </c>
       <c r="I247" s="4">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="J247" s="4"/>
       <c r="K247" s="4"/>
@@ -11876,7 +11714,7 @@
         <v>7</v>
       </c>
       <c r="I248" s="2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J248" s="2" t="s">
         <v>44</v>
@@ -11895,7 +11733,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="249" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A249" s="4">
         <v>130</v>
       </c>
@@ -11910,9 +11748,7 @@
       <c r="F249" s="4"/>
       <c r="G249" s="4"/>
       <c r="H249" s="4"/>
-      <c r="I249" s="4">
-        <v>0</v>
-      </c>
+      <c r="I249" s="4"/>
       <c r="J249" s="4">
         <v>2</v>
       </c>
@@ -11962,7 +11798,7 @@
         <v>3</v>
       </c>
       <c r="I250" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J250" s="2"/>
       <c r="K250" s="2"/>
@@ -11979,7 +11815,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="251" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A251" s="4">
         <v>132</v>
       </c>
@@ -11994,9 +11830,7 @@
       <c r="F251" s="4"/>
       <c r="G251" s="4"/>
       <c r="H251" s="4"/>
-      <c r="I251" s="4">
-        <v>0</v>
-      </c>
+      <c r="I251" s="4"/>
       <c r="J251" s="4">
         <v>0</v>
       </c>
@@ -12046,7 +11880,7 @@
         <v>26</v>
       </c>
       <c r="I252" s="2">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="J252" s="3">
         <v>46276</v>
@@ -12093,7 +11927,7 @@
         <v>20</v>
       </c>
       <c r="I253" s="4">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J253" s="4"/>
       <c r="K253" s="4"/>
@@ -12136,7 +11970,7 @@
         <v>36</v>
       </c>
       <c r="I254" s="2">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="J254" s="2"/>
       <c r="K254" s="2"/>
@@ -12181,7 +12015,7 @@
         <v>3</v>
       </c>
       <c r="I255" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J255" s="4"/>
       <c r="K255" s="4"/>
@@ -12198,7 +12032,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="256" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A256" s="2">
         <v>137</v>
       </c>
@@ -12213,9 +12047,7 @@
       <c r="F256" s="2"/>
       <c r="G256" s="2"/>
       <c r="H256" s="2"/>
-      <c r="I256" s="2">
-        <v>0</v>
-      </c>
+      <c r="I256" s="2"/>
       <c r="J256" s="2">
         <v>2</v>
       </c>
@@ -12265,7 +12097,7 @@
         <v>35</v>
       </c>
       <c r="I257" s="4">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="J257" s="5">
         <v>46339</v>
@@ -12310,7 +12142,7 @@
         <v>3</v>
       </c>
       <c r="I258" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J258" s="2"/>
       <c r="K258" s="2"/>
@@ -12353,7 +12185,7 @@
         <v>40</v>
       </c>
       <c r="I259" s="4">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J259" s="4"/>
       <c r="K259" s="5">
@@ -12372,7 +12204,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="260" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A260" s="2">
         <v>141</v>
       </c>
@@ -12387,9 +12219,7 @@
       <c r="F260" s="2"/>
       <c r="G260" s="2"/>
       <c r="H260" s="2"/>
-      <c r="I260" s="2">
-        <v>0</v>
-      </c>
+      <c r="I260" s="2"/>
       <c r="J260" s="2">
         <v>2</v>
       </c>
@@ -12439,7 +12269,7 @@
         <v>3</v>
       </c>
       <c r="I261" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J261" s="4"/>
       <c r="K261" s="4"/>
@@ -12456,7 +12286,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="262" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A262" s="2">
         <v>143</v>
       </c>
@@ -12471,9 +12301,7 @@
       <c r="F262" s="2"/>
       <c r="G262" s="2"/>
       <c r="H262" s="2"/>
-      <c r="I262" s="2">
-        <v>0</v>
-      </c>
+      <c r="I262" s="2"/>
       <c r="J262" s="2">
         <v>0</v>
       </c>
@@ -12523,7 +12351,7 @@
         <v>27</v>
       </c>
       <c r="I263" s="4">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="J263" s="5">
         <v>46276</v>
@@ -12570,7 +12398,7 @@
         <v>22</v>
       </c>
       <c r="I264" s="2">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="J264" s="3">
         <v>46339</v>
@@ -12615,7 +12443,7 @@
         <v>36</v>
       </c>
       <c r="I265" s="4">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="J265" s="5">
         <v>46243</v>
@@ -12634,7 +12462,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="266" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A266" s="2">
         <v>147</v>
       </c>
@@ -12649,9 +12477,7 @@
       <c r="F266" s="2"/>
       <c r="G266" s="2"/>
       <c r="H266" s="2"/>
-      <c r="I266" s="2">
-        <v>0</v>
-      </c>
+      <c r="I266" s="2"/>
       <c r="J266" s="2">
         <v>5</v>
       </c>
@@ -12701,7 +12527,7 @@
         <v>3</v>
       </c>
       <c r="I267" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J267" s="4"/>
       <c r="K267" s="4"/>
@@ -12744,7 +12570,7 @@
         <v>30</v>
       </c>
       <c r="I268" s="2">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J268" s="3">
         <v>46339</v>
@@ -12789,7 +12615,7 @@
         <v>11</v>
       </c>
       <c r="I269" s="4">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J269" s="5">
         <v>46276</v>
@@ -12808,7 +12634,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="270" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A270" s="2">
         <v>151</v>
       </c>
@@ -12823,9 +12649,7 @@
       <c r="F270" s="2"/>
       <c r="G270" s="2"/>
       <c r="H270" s="2"/>
-      <c r="I270" s="2">
-        <v>0</v>
-      </c>
+      <c r="I270" s="2"/>
       <c r="J270" s="2">
         <v>4</v>
       </c>
@@ -12875,7 +12699,7 @@
         <v>40</v>
       </c>
       <c r="I271" s="4">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J271" s="4"/>
       <c r="K271" s="4"/>
@@ -12894,7 +12718,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="272" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A272" s="2">
         <v>153</v>
       </c>
@@ -12909,9 +12733,7 @@
       <c r="F272" s="2"/>
       <c r="G272" s="2"/>
       <c r="H272" s="2"/>
-      <c r="I272" s="2">
-        <v>0</v>
-      </c>
+      <c r="I272" s="2"/>
       <c r="J272" s="2">
         <v>0</v>
       </c>
@@ -12961,7 +12783,7 @@
         <v>40</v>
       </c>
       <c r="I273" s="4">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J273" s="4"/>
       <c r="K273" s="5">
@@ -12980,7 +12802,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="274" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A274" s="2">
         <v>155</v>
       </c>
@@ -12995,9 +12817,7 @@
       <c r="F274" s="2"/>
       <c r="G274" s="2"/>
       <c r="H274" s="2"/>
-      <c r="I274" s="2">
-        <v>0</v>
-      </c>
+      <c r="I274" s="2"/>
       <c r="J274" s="2">
         <v>0</v>
       </c>
@@ -13047,7 +12867,7 @@
         <v>28</v>
       </c>
       <c r="I275" s="4">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="J275" s="5">
         <v>46276</v>
@@ -13094,7 +12914,7 @@
         <v>9</v>
       </c>
       <c r="I276" s="2">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J276" s="2" t="s">
         <v>44</v>
@@ -13141,7 +12961,7 @@
         <v>3</v>
       </c>
       <c r="I277" s="4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J277" s="4"/>
       <c r="K277" s="4"/>
@@ -13184,7 +13004,7 @@
         <v>40</v>
       </c>
       <c r="I278" s="2">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J278" s="2"/>
       <c r="K278" s="2" t="s">
@@ -13229,7 +13049,7 @@
         <v>40</v>
       </c>
       <c r="I279" s="4">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J279" s="4"/>
       <c r="K279" s="4"/>
@@ -13272,7 +13092,7 @@
         <v>40</v>
       </c>
       <c r="I280" s="2">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J280" s="2"/>
       <c r="K280" s="2"/>
@@ -13353,9 +13173,7 @@
         <v>22</v>
       </c>
       <c r="H282" s="2"/>
-      <c r="I282" s="2">
-        <v>0</v>
-      </c>
+      <c r="I282" s="2"/>
       <c r="J282" s="2"/>
       <c r="K282" s="2"/>
       <c r="L282" s="2"/>
@@ -13397,7 +13215,7 @@
         <v>13</v>
       </c>
       <c r="I283" s="4">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J283" s="4"/>
       <c r="K283" s="4"/>
@@ -13440,7 +13258,7 @@
         <v>13</v>
       </c>
       <c r="I284" s="2">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J284" s="2"/>
       <c r="K284" s="2"/>
@@ -13483,7 +13301,7 @@
         <v>13</v>
       </c>
       <c r="I285" s="4">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J285" s="4"/>
       <c r="K285" s="4"/>
@@ -13526,7 +13344,7 @@
         <v>13</v>
       </c>
       <c r="I286" s="2">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="J286" s="2"/>
       <c r="K286" s="2"/>
@@ -13569,7 +13387,7 @@
         <v>20</v>
       </c>
       <c r="I287" s="4">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J287" s="4"/>
       <c r="K287" s="4"/>
@@ -13612,7 +13430,7 @@
         <v>20</v>
       </c>
       <c r="I288" s="2">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J288" s="2"/>
       <c r="K288" s="2"/>
@@ -13655,7 +13473,7 @@
         <v>11</v>
       </c>
       <c r="I289" s="4">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J289" s="5">
         <v>46338</v>
@@ -13698,7 +13516,7 @@
         <v>11</v>
       </c>
       <c r="I290" s="2">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J290" s="3">
         <v>46369</v>
@@ -13741,7 +13559,7 @@
         <v>9</v>
       </c>
       <c r="I291" s="4">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J291" s="4"/>
       <c r="K291" s="4"/>
@@ -13784,7 +13602,7 @@
         <v>30</v>
       </c>
       <c r="I292" s="2">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J292" s="2"/>
       <c r="K292" s="2"/>
@@ -13827,7 +13645,7 @@
         <v>17</v>
       </c>
       <c r="I293" s="4">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="J293" s="4" t="s">
         <v>33</v>
@@ -13870,7 +13688,7 @@
         <v>16</v>
       </c>
       <c r="I294" s="2">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="J294" s="2" t="s">
         <v>44</v>
@@ -13913,7 +13731,7 @@
         <v>6</v>
       </c>
       <c r="I295" s="4">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J295" s="4"/>
       <c r="K295" s="4"/>
@@ -13956,7 +13774,7 @@
         <v>5</v>
       </c>
       <c r="I296" s="2">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J296" s="2"/>
       <c r="K296" s="2"/>
@@ -13999,7 +13817,7 @@
         <v>40</v>
       </c>
       <c r="I297" s="4">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J297" s="4"/>
       <c r="K297" s="5">
@@ -14042,7 +13860,7 @@
         <v>40</v>
       </c>
       <c r="I298" s="2">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J298" s="3">
         <v>46212</v>
@@ -14085,7 +13903,7 @@
         <v>30</v>
       </c>
       <c r="I299" s="4">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J299" s="4"/>
       <c r="K299" s="4"/>
@@ -14128,7 +13946,7 @@
         <v>10</v>
       </c>
       <c r="I300" s="2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J300" s="2"/>
       <c r="K300" s="2"/>
@@ -14173,7 +13991,7 @@
         <v>9</v>
       </c>
       <c r="I301" s="4">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J301" s="4"/>
       <c r="K301" s="4" t="s">
@@ -14215,9 +14033,7 @@
         <v>22</v>
       </c>
       <c r="H302" s="2"/>
-      <c r="I302" s="2">
-        <v>0</v>
-      </c>
+      <c r="I302" s="2"/>
       <c r="J302" s="2"/>
       <c r="K302" s="2"/>
       <c r="L302" s="3">
@@ -14259,7 +14075,7 @@
         <v>15</v>
       </c>
       <c r="I303" s="4">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J303" s="4"/>
       <c r="K303" s="4"/>
@@ -14304,7 +14120,7 @@
         <v>23</v>
       </c>
       <c r="I304" s="2">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="J304" s="3">
         <v>46339</v>
@@ -14349,7 +14165,7 @@
         <v>11</v>
       </c>
       <c r="I305" s="4">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J305" s="5">
         <v>46211</v>
@@ -14478,7 +14294,7 @@
         <v>30</v>
       </c>
       <c r="I308" s="2">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J308" s="2"/>
       <c r="K308" s="2"/>
@@ -14521,7 +14337,7 @@
         <v>23</v>
       </c>
       <c r="I309" s="4">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="J309" s="4"/>
       <c r="K309" s="4" t="s">
@@ -14566,7 +14382,7 @@
         <v>24</v>
       </c>
       <c r="I310" s="2">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="J310" s="2"/>
       <c r="K310" s="3">
@@ -14611,7 +14427,7 @@
         <v>22</v>
       </c>
       <c r="I311" s="4">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="J311" s="4"/>
       <c r="K311" s="5">
@@ -14630,7 +14446,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="312" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A312" s="2">
         <v>193</v>
       </c>
@@ -14645,9 +14461,7 @@
       <c r="F312" s="2"/>
       <c r="G312" s="2"/>
       <c r="H312" s="2"/>
-      <c r="I312" s="2">
-        <v>0</v>
-      </c>
+      <c r="I312" s="2"/>
       <c r="J312" s="2">
         <v>15</v>
       </c>
@@ -14694,9 +14508,7 @@
         <v>22</v>
       </c>
       <c r="H313" s="4"/>
-      <c r="I313" s="4">
-        <v>0</v>
-      </c>
+      <c r="I313" s="4"/>
       <c r="J313" s="4"/>
       <c r="K313" s="4"/>
       <c r="L313" s="4" t="s">
@@ -14739,9 +14551,7 @@
         <v>22</v>
       </c>
       <c r="H314" s="2"/>
-      <c r="I314" s="2">
-        <v>0</v>
-      </c>
+      <c r="I314" s="2"/>
       <c r="J314" s="2"/>
       <c r="K314" s="2"/>
       <c r="L314" s="2"/>
@@ -14780,9 +14590,7 @@
         <v>22</v>
       </c>
       <c r="H315" s="4"/>
-      <c r="I315" s="4">
-        <v>0</v>
-      </c>
+      <c r="I315" s="4"/>
       <c r="J315" s="4"/>
       <c r="K315" s="4" t="s">
         <v>33</v>
@@ -14798,7 +14606,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="316" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A316" s="2">
         <v>197</v>
       </c>
@@ -14813,9 +14621,7 @@
       <c r="F316" s="2"/>
       <c r="G316" s="2"/>
       <c r="H316" s="2"/>
-      <c r="I316" s="2">
-        <v>0</v>
-      </c>
+      <c r="I316" s="2"/>
       <c r="J316" s="2">
         <v>0</v>
       </c>
@@ -14862,9 +14668,7 @@
         <v>22</v>
       </c>
       <c r="H317" s="4"/>
-      <c r="I317" s="4">
-        <v>0</v>
-      </c>
+      <c r="I317" s="4"/>
       <c r="J317" s="4"/>
       <c r="K317" s="5">
         <v>46212</v>
@@ -14903,9 +14707,7 @@
         <v>22</v>
       </c>
       <c r="H318" s="2"/>
-      <c r="I318" s="2">
-        <v>0</v>
-      </c>
+      <c r="I318" s="2"/>
       <c r="J318" s="2"/>
       <c r="K318" s="2"/>
       <c r="L318" s="2" t="s">
@@ -14921,7 +14723,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="319" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A319" s="4">
         <v>200</v>
       </c>
@@ -14936,9 +14738,7 @@
       <c r="F319" s="4"/>
       <c r="G319" s="4"/>
       <c r="H319" s="4"/>
-      <c r="I319" s="4">
-        <v>0</v>
-      </c>
+      <c r="I319" s="4"/>
       <c r="J319" s="4">
         <v>0</v>
       </c>
@@ -14988,7 +14788,7 @@
         <v>25</v>
       </c>
       <c r="I320" s="2">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="J320" s="3">
         <v>46276</v>
@@ -15035,7 +14835,7 @@
         <v>40</v>
       </c>
       <c r="I321" s="4">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J321" s="4"/>
       <c r="K321" s="4"/>
@@ -15052,7 +14852,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="322" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A322" s="2">
         <v>203</v>
       </c>
@@ -15067,9 +14867,7 @@
       <c r="F322" s="2"/>
       <c r="G322" s="2"/>
       <c r="H322" s="2"/>
-      <c r="I322" s="2">
-        <v>0</v>
-      </c>
+      <c r="I322" s="2"/>
       <c r="J322" s="2">
         <v>2</v>
       </c>
@@ -15119,7 +14917,7 @@
         <v>7</v>
       </c>
       <c r="I323" s="4">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J323" s="4"/>
       <c r="K323" s="4"/>
@@ -15162,7 +14960,7 @@
         <v>7</v>
       </c>
       <c r="I324" s="2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J324" s="2"/>
       <c r="K324" s="2"/>
@@ -15205,7 +15003,7 @@
         <v>7</v>
       </c>
       <c r="I325" s="4">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J325" s="4"/>
       <c r="K325" s="4"/>
@@ -15248,7 +15046,7 @@
         <v>7</v>
       </c>
       <c r="I326" s="2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J326" s="2"/>
       <c r="K326" s="2"/>
@@ -15291,7 +15089,7 @@
         <v>7</v>
       </c>
       <c r="I327" s="4">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J327" s="4"/>
       <c r="K327" s="4"/>
@@ -15334,7 +15132,7 @@
         <v>7</v>
       </c>
       <c r="I328" s="2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="J328" s="2"/>
       <c r="K328" s="2"/>
@@ -15377,7 +15175,7 @@
         <v>12</v>
       </c>
       <c r="I329" s="4">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J329" s="4"/>
       <c r="K329" s="4" t="s">
@@ -15420,7 +15218,7 @@
         <v>11</v>
       </c>
       <c r="I330" s="2">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J330" s="2"/>
       <c r="K330" s="2" t="s">
@@ -15463,7 +15261,7 @@
         <v>11</v>
       </c>
       <c r="I331" s="4">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="J331" s="4"/>
       <c r="K331" s="4" t="s">
@@ -15506,7 +15304,7 @@
         <v>9</v>
       </c>
       <c r="I332" s="2">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J332" s="2"/>
       <c r="K332" s="2"/>
@@ -15549,7 +15347,7 @@
         <v>8</v>
       </c>
       <c r="I333" s="4">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J333" s="4"/>
       <c r="K333" s="4"/>
@@ -15592,7 +15390,7 @@
         <v>8</v>
       </c>
       <c r="I334" s="2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J334" s="2"/>
       <c r="K334" s="2"/>
@@ -15635,7 +15433,7 @@
         <v>8</v>
       </c>
       <c r="I335" s="4">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J335" s="4"/>
       <c r="K335" s="4"/>
@@ -15678,7 +15476,7 @@
         <v>15</v>
       </c>
       <c r="I336" s="2">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J336" s="2"/>
       <c r="K336" s="2"/>
@@ -15721,7 +15519,7 @@
         <v>15</v>
       </c>
       <c r="I337" s="4">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J337" s="4"/>
       <c r="K337" s="4"/>
@@ -15764,7 +15562,7 @@
         <v>12</v>
       </c>
       <c r="I338" s="2">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="J338" s="2"/>
       <c r="K338" s="2"/>
@@ -15781,7 +15579,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="339" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A339" s="4">
         <v>220</v>
       </c>
@@ -15796,9 +15594,7 @@
       <c r="F339" s="4"/>
       <c r="G339" s="4"/>
       <c r="H339" s="4"/>
-      <c r="I339" s="4">
-        <v>0</v>
-      </c>
+      <c r="I339" s="4"/>
       <c r="J339" s="4">
         <v>0</v>
       </c>
@@ -15848,7 +15644,7 @@
         <v>3</v>
       </c>
       <c r="I340" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J340" s="2"/>
       <c r="K340" s="2"/>
@@ -15891,7 +15687,7 @@
         <v>36</v>
       </c>
       <c r="I341" s="4">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="J341" s="4"/>
       <c r="K341" s="4"/>
@@ -15936,7 +15732,7 @@
         <v>3</v>
       </c>
       <c r="I342" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J342" s="2"/>
       <c r="K342" s="2"/>
@@ -15953,7 +15749,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="343" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A343" s="4">
         <v>224</v>
       </c>
@@ -15968,9 +15764,7 @@
       <c r="F343" s="4"/>
       <c r="G343" s="4"/>
       <c r="H343" s="4"/>
-      <c r="I343" s="4">
-        <v>0</v>
-      </c>
+      <c r="I343" s="4"/>
       <c r="J343" s="4">
         <v>0</v>
       </c>
@@ -16020,7 +15814,7 @@
         <v>40</v>
       </c>
       <c r="I344" s="2">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J344" s="2"/>
       <c r="K344" s="3">
@@ -16065,7 +15859,7 @@
         <v>48</v>
       </c>
       <c r="I345" s="4">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="J345" s="5">
         <v>46339</v>
@@ -16086,7 +15880,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="346" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A346" s="2">
         <v>227</v>
       </c>
@@ -16101,9 +15895,7 @@
       <c r="F346" s="2"/>
       <c r="G346" s="2"/>
       <c r="H346" s="2"/>
-      <c r="I346" s="2">
-        <v>0</v>
-      </c>
+      <c r="I346" s="2"/>
       <c r="J346" s="2">
         <v>2</v>
       </c>
@@ -16153,7 +15945,7 @@
         <v>26</v>
       </c>
       <c r="I347" s="4">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="J347" s="5">
         <v>46276</v>
@@ -16174,7 +15966,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="348" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A348" s="2">
         <v>229</v>
       </c>
@@ -16189,9 +15981,7 @@
       <c r="F348" s="2"/>
       <c r="G348" s="2"/>
       <c r="H348" s="2"/>
-      <c r="I348" s="2">
-        <v>0</v>
-      </c>
+      <c r="I348" s="2"/>
       <c r="J348" s="2">
         <v>2</v>
       </c>
@@ -16241,7 +16031,7 @@
         <v>40</v>
       </c>
       <c r="I349" s="4">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J349" s="5">
         <v>46276</v>
@@ -16283,9 +16073,7 @@
         <v>22</v>
       </c>
       <c r="H350" s="2"/>
-      <c r="I350" s="2">
-        <v>0</v>
-      </c>
+      <c r="I350" s="2"/>
       <c r="J350" s="2"/>
       <c r="K350" s="2"/>
       <c r="L350" s="2"/>
@@ -16327,7 +16115,7 @@
         <v>19</v>
       </c>
       <c r="I351" s="4">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="J351" s="4"/>
       <c r="K351" s="4"/>
@@ -16374,7 +16162,7 @@
         <v>4</v>
       </c>
       <c r="I352" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J352" s="2"/>
       <c r="K352" s="2"/>
@@ -16391,7 +16179,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="353" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="353" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A353" s="4">
         <v>234</v>
       </c>
@@ -16406,9 +16194,7 @@
       <c r="F353" s="4"/>
       <c r="G353" s="4"/>
       <c r="H353" s="4"/>
-      <c r="I353" s="4">
-        <v>0</v>
-      </c>
+      <c r="I353" s="4"/>
       <c r="J353" s="4">
         <v>2</v>
       </c>
@@ -16455,9 +16241,7 @@
         <v>22</v>
       </c>
       <c r="H354" s="2"/>
-      <c r="I354" s="2">
-        <v>0</v>
-      </c>
+      <c r="I354" s="2"/>
       <c r="J354" s="2"/>
       <c r="K354" s="2"/>
       <c r="L354" s="2"/>
@@ -16496,9 +16280,7 @@
         <v>22</v>
       </c>
       <c r="H355" s="4"/>
-      <c r="I355" s="4">
-        <v>0</v>
-      </c>
+      <c r="I355" s="4"/>
       <c r="J355" s="4"/>
       <c r="K355" s="4"/>
       <c r="L355" s="4"/>
@@ -16540,7 +16322,7 @@
         <v>21</v>
       </c>
       <c r="I356" s="2">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="J356" s="2"/>
       <c r="K356" s="2"/>
@@ -16585,7 +16367,7 @@
         <v>31</v>
       </c>
       <c r="I357" s="4">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="J357" s="5">
         <v>46339</v>
@@ -16604,7 +16386,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="358" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="358" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A358" s="2">
         <v>239</v>
       </c>
@@ -16619,9 +16401,7 @@
       <c r="F358" s="2"/>
       <c r="G358" s="2"/>
       <c r="H358" s="2"/>
-      <c r="I358" s="2">
-        <v>0</v>
-      </c>
+      <c r="I358" s="2"/>
       <c r="J358" s="2">
         <v>2</v>
       </c>
@@ -16671,7 +16451,7 @@
         <v>22</v>
       </c>
       <c r="I359" s="4">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="J359" s="4"/>
       <c r="K359" s="4" t="s">
@@ -16688,7 +16468,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="360" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="360" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A360" s="2">
         <v>241</v>
       </c>
@@ -16703,9 +16483,7 @@
       <c r="F360" s="2"/>
       <c r="G360" s="2"/>
       <c r="H360" s="2"/>
-      <c r="I360" s="2">
-        <v>0</v>
-      </c>
+      <c r="I360" s="2"/>
       <c r="J360" s="2">
         <v>0</v>
       </c>
@@ -16755,7 +16533,7 @@
         <v>40</v>
       </c>
       <c r="I361" s="4">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J361" s="4"/>
       <c r="K361" s="4"/>
@@ -16798,7 +16576,7 @@
         <v>40</v>
       </c>
       <c r="I362" s="2">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="J362" s="2"/>
       <c r="K362" s="2"/>
@@ -16841,7 +16619,7 @@
         <v>24</v>
       </c>
       <c r="I363" s="4">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="J363" s="5">
         <v>46212</v>
@@ -16884,7 +16662,7 @@
         <v>23</v>
       </c>
       <c r="I364" s="2">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="J364" s="2"/>
       <c r="K364" s="2"/>
@@ -16901,7 +16679,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="365" spans="1:17" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="365" spans="1:17" ht="57.6" hidden="1" x14ac:dyDescent="0.3">
       <c r="A365" s="4">
         <v>246</v>
       </c>
@@ -16943,6 +16721,139 @@
       <c r="Q365" s="4"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:Q365" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="AGRICULTURA ECOLOGICA (AGRD600)"/>
+        <filter val="AGROCOMERCIO (AGRD761)"/>
+        <filter val="AGROINDUSTRIAS (AGRD412)"/>
+        <filter val="AGROPLASTICULTURA (AGRD700)"/>
+        <filter val="ALGEBRA LINEAL (MATD113)"/>
+        <filter val="ANALISIS INSTRUMENTAL (IQMD452)"/>
+        <filter val="ANALISIS INSTRUMENTAL Y DE ALIMENTOS (AGRD354)"/>
+        <filter val="ASEGURAMIENTO ESTADISTICO DE LA CALIDAD (AGRD842)"/>
+        <filter val="BALANCE DE ENERGIA (IAQD423)"/>
+        <filter val="BALANCE DE MASA (IAQD323)"/>
+        <filter val="BIOINGENIERIA (AGRD723)"/>
+        <filter val="BIOLOGIA (IAQD462)"/>
+        <filter val="BIOQUIMICA (IAQD562)"/>
+        <filter val="CALCULO EN UNA VARIABLE (MATD123)"/>
+        <filter val="CONTROL DE LA CONTAMINACION ATMOSFERICA Y EFLUENTES LIQUIDOS (IQMD802)"/>
+        <filter val="DISEÑO DE BIOPROCESOS (IQMD901)"/>
+        <filter val="DISEÑO DE PLANTAS (IQMD814)"/>
+        <filter val="DISEÑO DE PLANTAS AGROINDUSTRIALES (AGRD814)"/>
+        <filter val="DISEÑO DE PLANTAS METALURGICAS (IQMD903)"/>
+        <filter val="DISEÑO DE TRABAJO DE INTEGRACION CURRICULAR / PREPARACION EXAMEN DE CARACTER COMPLEXIVO (TITD101)"/>
+        <filter val="ECOLOGIA Y AMBIENTE (AMBD900)"/>
+        <filter val="ECUACIONES DIFERENCIALES ORDINARIAS (MATD213)"/>
+        <filter val="EVALUACION DE IMPACTO Y AUDITORIA AMBIENTAL (IAQD722)"/>
+        <filter val="FISICA PARA INGENIERIA (IAQD242)"/>
+        <filter val="FISICOQUIMICA (IQMD653)"/>
+        <filter val="FORMULACION Y EVALUACION DE PROYECTOS (ADMD800)"/>
+        <filter val="GERENCIA DE OPERACIONES (IQMD752)"/>
+        <filter val="GESTION DE PROCESOS Y CALIDAD (ADMD611)"/>
+        <filter val="GESTION ORGANIZACIONAL (ADMD511)"/>
+        <filter val="HERRAMIENTAS INFORMATICAS (ICOD111)"/>
+        <filter val="INGENIERIA DE ALIMENTOS (AGRD733)"/>
+        <filter val="INGENIERIA DE LA REACCION I (IQMD733)"/>
+        <filter val="INGENIERIA DE LA REACCION II (IQMD832)"/>
+        <filter val="INGENIERIA FINANCIERA (ADMD711)"/>
+        <filter val="INGLES (IEXD200)"/>
+        <filter val="INTRODUCCION A LA PRODUCCION ANIMAL (AGRD563)"/>
+        <filter val="INTRODUCCION A LA PRODUCCION VEGETAL (AGRD553)"/>
+        <filter val="INTRODUCCION A LA TECNOLOGIA DEL PETROLEO (IQMD602)"/>
+        <filter val="LABORATORIO ANALISIS INSTRUMENTAL (IQMD452L)"/>
+        <filter val="LABORATORIO ANALISIS INSTRUMENTAL Y DE ALIMENTOS (AGRD354L)"/>
+        <filter val="LABORATORIO BIOINGENIERIA (AGRD723L)"/>
+        <filter val="LABORATORIO BIOQUIMICA (IAQD562L)"/>
+        <filter val="LABORATORIO CONTROL DE LA CONTAMINACION ATMOSFERICA Y EFLUEN (IQMD802L)"/>
+        <filter val="LABORATORIO FISICOQUIMICA (IQMD653L)"/>
+        <filter val="LABORATORIO INGENIERIA DE ALIMENTOS (AGRD733L)"/>
+        <filter val="LABORATORIO INGENIERIA DE LA REACCION II (IQMD832L)"/>
+        <filter val="LABORATORIO INTRODUCCION A LA PRODUCCION ANIMAL (AGRD563L)"/>
+        <filter val="LABORATORIO MANEJO DE RESIDUOS SOLIDOS Y SISTEMAS DE GERENCI (IQMD902L)"/>
+        <filter val="LABORATORIO MANEJO DE SUELOS AGRICOLAS (AGRD453L)"/>
+        <filter val="LABORATORIO MECANICA DE FLUIDOS (AGRD522L)"/>
+        <filter val="LABORATORIO MECANICA DE FLUIDOS I (IQMD523L)"/>
+        <filter val="LABORATORIO MECANICA DE FLUIDOS II (IQMD623L)"/>
+        <filter val="LABORATORIO MECANICA NEWTONIANA (FISD134L)"/>
+        <filter val="LABORATORIO METALURGIA EXTRACTIVA (IQMD803L)"/>
+        <filter val="LABORATORIO MICROBIOLOGIA INDUSTRIAL Y DE ALIMENTOS (AGRD623L)"/>
+        <filter val="LABORATORIO MICROBIOLOGIA INDUSTRIAL Y PRESERVACION DE ALIME (IQMD801L)"/>
+        <filter val="LABORATORIO MODELADO Y CONTROL AUTOMATICO (IQMD743L)"/>
+        <filter val="LABORATORIO OPERACIONES UNITARIAS AGROINDUSTRIALES (AGRD613L)"/>
+        <filter val="LABORATORIO OPERACIONES UNITARIAS I (IQMD613L)"/>
+        <filter val="LABORATORIO OPERACIONES UNITARIAS II (IQMD713L)"/>
+        <filter val="LABORATORIO POLIMEROS EN LA AGROINDUSTRIA (AGRD743L)"/>
+        <filter val="LABORATORIO POSCOSECHA (AGRD752L)"/>
+        <filter val="LABORATORIO PRODUCCION ANIMAL (AGRD643L)"/>
+        <filter val="LABORATORIO PRODUCCION VEGETAL (AGRD633L)"/>
+        <filter val="LABORATORIO PRODUCTOS NO ALIMENTICIOS I (AGRD803L)"/>
+        <filter val="LABORATORIO PROGRAMACION (IAQD262L)"/>
+        <filter val="LABORATORIO QUIMICA ANALITICA (IQMD354L)"/>
+        <filter val="LABORATORIO QUIMICA BIOORGANICA (AGRD443L)"/>
+        <filter val="LABORATORIO QUIMICA ORGANICA I (IAQD343L)"/>
+        <filter val="LABORATORIO QUIMICA ORGANICA II (IQMD443L)"/>
+        <filter val="LABORATORIO TECNOLOGIA DE ALIMENTOS I (AGRD801L)"/>
+        <filter val="LABORATORIO TERMODINAMICA II (IAQD432L)"/>
+        <filter val="LABORATORIO TRANSFERENCIA DE CALOR I (IQMD533L)"/>
+        <filter val="LABORATORIO TRANSFERENCIA DE CALOR II (IQMD633L)"/>
+        <filter val="LABORATORIO TRANSFERENCIA DE MASA I (IQMD543L)"/>
+        <filter val="LABORATORIO TRANSFERENCIA DE MASA II (IQMD643L)"/>
+        <filter val="LABORATORIO TRANSFERENCIA DE MASA Y CALOR (AGRD534L)"/>
+        <filter val="MANEJO DE RESIDUOS SOLIDOS Y SISTEMAS DE GERENCIAMIENTO AMBIENTAL (IQMD902)"/>
+        <filter val="MANEJO DE SUELOS AGRICOLAS (AGRD453)"/>
+        <filter val="MATEMATICA APLICADA EN INGENIERIA I (IAQD222)"/>
+        <filter val="MATEMATICA APLICADA EN INGENIERIA II (IAQD312)"/>
+        <filter val="MATERIALES PARA INGENIERIA Y CORROSION (IQMD552)"/>
+        <filter val="MECANICA DE FLUIDOS (AGRD522)"/>
+        <filter val="MECANICA DE FLUIDOS I (IQMD523)"/>
+        <filter val="MECANICA DE FLUIDOS II (IQMD623)"/>
+        <filter val="MECANICA NEWTONIANA (FISD134)"/>
+        <filter val="MERCADEO Y VENTAS (IQMD810)"/>
+        <filter val="METALURGIA EXTRACTIVA (IQMD803)"/>
+        <filter val="MICROBIOLOGIA INDUSTRIAL Y DE ALIMENTOS (AGRD623)"/>
+        <filter val="MICROBIOLOGIA INDUSTRIAL Y PRESERVACION DE ALIMENTOS (IQMD801)"/>
+        <filter val="MODELADO Y CONTROL AUTOMATICO (IQMD743)"/>
+        <filter val="OPERACIONES UNITARIAS AGROINDUSTRIALES (AGRD613)"/>
+        <filter val="OPERACIONES UNITARIAS I (IQMD613)"/>
+        <filter val="OPERACIONES UNITARIAS II (IQMD713)"/>
+        <filter val="POLIMEROS EN LA AGROINDUSTRIA (AGRD743)"/>
+        <filter val="POSCOSECHA (AGRD752)"/>
+        <filter val="PRACTICAS DE SERVICIO COMUNITARIO (PSCD202)"/>
+        <filter val="PRACTICAS LABORALES (PRLD105)"/>
+        <filter val="PROBABILIDAD Y ESTADISTICA BASICAS (MATD223)"/>
+        <filter val="PRODUCCION ANIMAL (AGRD643)"/>
+        <filter val="PRODUCCION VEGETAL (AGRD633)"/>
+        <filter val="PRODUCTOS NO ALIMENTICIOS I (AGRD803)"/>
+        <filter val="PRODUCTOS NO ALIMENTICIOS II (AGRD903)"/>
+        <filter val="PROGRAMACION (IAQD262)"/>
+        <filter val="QUIMICA ANALITICA (IQMD354)"/>
+        <filter val="QUIMICA AVANZADA (IAQD253)"/>
+        <filter val="QUIMICA BIOORGANICA (AGRD443)"/>
+        <filter val="QUIMICA GENERAL (QUID143)"/>
+        <filter val="QUIMICA INDUSTRIAL (IQMD412)"/>
+        <filter val="QUIMICA ORGANICA I (IAQD343)"/>
+        <filter val="QUIMICA ORGANICA II (IQMD443)"/>
+        <filter val="RADIOQUIMICA (IQMD601)"/>
+        <filter val="SEGURIDAD INDUSTRIAL Y SALUD OCUPACIONAL (IAQD511)"/>
+        <filter val="SIMULACION DE PROCESOS AGROINDUSTRIALES (AGRD822)"/>
+        <filter val="SIMULACION DE PROCESOS QUIMICOS (IQMD822)"/>
+        <filter val="SUBPRODUCTOS AGROINDUSTRIALES (AGRD810)"/>
+        <filter val="TECNOLOGIA DE ALIMENTOS I (AGRD801)"/>
+        <filter val="TECNOLOGIA DE POLIMEROS (IQMD603)"/>
+        <filter val="TECNOLOGIA TEXTIL (IQMD703)"/>
+        <filter val="TERMODINAMICA I (IAQD333)"/>
+        <filter val="TERMODINAMICA II (IAQD432)"/>
+        <filter val="TRABAJO DE INTEGRACION CURRICULAR/EXAMEN DE CARACTER COMPLEXIVO (TITD201)"/>
+        <filter val="TRANSFERENCIA DE CALOR I (IQMD533)"/>
+        <filter val="TRANSFERENCIA DE CALOR II (IQMD633)"/>
+        <filter val="TRANSFERENCIA DE MASA I (IQMD543)"/>
+        <filter val="TRANSFERENCIA DE MASA II (IQMD643)"/>
+        <filter val="TRANSFERENCIA DE MASA Y CALOR (AGRD534)"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>